<commit_message>
link for tickets added
</commit_message>
<xml_diff>
--- a/UConnBleedBlue/wwwroot/players/Players.xlsx
+++ b/UConnBleedBlue/wwwroot/players/Players.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repos\UConnBleedBlue\UConnBleedBlue\wwwroot\players\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{47AF074A-E916-46B9-B1C4-74089F55E6D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{391DE659-D108-454A-A60E-0B8F84E79AF4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2730" yWindow="2730" windowWidth="21600" windowHeight="11295" xr2:uid="{4F83266A-41F9-4FA3-9290-1EB5622BBFC1}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{4F83266A-41F9-4FA3-9290-1EB5622BBFC1}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="68">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="114">
   <si>
     <t>Demers, Kenny</t>
   </si>
@@ -240,6 +240,144 @@
   </si>
   <si>
     <t>dennis.p.oconnell@gmail.com</t>
+  </si>
+  <si>
+    <t>Nesteruk, Warren</t>
+  </si>
+  <si>
+    <t>hef714@aol.com</t>
+  </si>
+  <si>
+    <t>O'Roark, Mike</t>
+  </si>
+  <si>
+    <t>mikeoroark23@gmail.com</t>
+  </si>
+  <si>
+    <t>Henrich, Joe</t>
+  </si>
+  <si>
+    <t>jhenrich1972@gmail.com</t>
+  </si>
+  <si>
+    <t>Torre, Joe</t>
+  </si>
+  <si>
+    <t>jtorre2829@gmail.com</t>
+  </si>
+  <si>
+    <t>Mack, Gary</t>
+  </si>
+  <si>
+    <t>g.mack96@yahoo.com</t>
+  </si>
+  <si>
+    <t>Marrus, Glenn</t>
+  </si>
+  <si>
+    <t>Gjhusky52@yahoo.com</t>
+  </si>
+  <si>
+    <t>s.vibberts@yahoo.com</t>
+  </si>
+  <si>
+    <t>oldparsonage3@gmail.com</t>
+  </si>
+  <si>
+    <t>Petrillo, Peter</t>
+  </si>
+  <si>
+    <t>Lane, Peter</t>
+  </si>
+  <si>
+    <t>Peterlane@optonline.net</t>
+  </si>
+  <si>
+    <t>Anglim, Patrick</t>
+  </si>
+  <si>
+    <t>patrick@drpflexpak.com</t>
+  </si>
+  <si>
+    <t>Berry, Craig</t>
+  </si>
+  <si>
+    <t>cwb84122@gmail.com</t>
+  </si>
+  <si>
+    <t>Myers, Norm</t>
+  </si>
+  <si>
+    <t>Npmyers@sbcglobal.net</t>
+  </si>
+  <si>
+    <t>timarmour.ycn@gmail.com</t>
+  </si>
+  <si>
+    <t>shbrann52@gmail.com</t>
+  </si>
+  <si>
+    <t>coachcorreia7@gmail.com</t>
+  </si>
+  <si>
+    <t>cordseller1@gmail.com</t>
+  </si>
+  <si>
+    <t>kpdemers073@gmail.com</t>
+  </si>
+  <si>
+    <t>marksflood1@gmail.com</t>
+  </si>
+  <si>
+    <t>gragmgorski@yahoo.com</t>
+  </si>
+  <si>
+    <t>robertinnis@yahoo.com</t>
+  </si>
+  <si>
+    <t>plamagna1@nefitness.com</t>
+  </si>
+  <si>
+    <t>mludwig67@optonline.net</t>
+  </si>
+  <si>
+    <t>pmargiatto66@gmail.com</t>
+  </si>
+  <si>
+    <t>marcmof@me.com</t>
+  </si>
+  <si>
+    <t>tomjney@yahoo.com</t>
+  </si>
+  <si>
+    <t>Miller, Ken</t>
+  </si>
+  <si>
+    <t>Kmills8080@gmail.com</t>
+  </si>
+  <si>
+    <t>bobnichols49@gmail.com</t>
+  </si>
+  <si>
+    <t>pnwokeji@hotmail.com</t>
+  </si>
+  <si>
+    <t>jpass33@earthlink.net</t>
+  </si>
+  <si>
+    <t>craigprimiani@aol.com</t>
+  </si>
+  <si>
+    <t>rick.robustelli@gmail.com</t>
+  </si>
+  <si>
+    <t>ralphtiner83@gmail.com</t>
+  </si>
+  <si>
+    <t>Murphy, Dan</t>
+  </si>
+  <si>
+    <t>Dmurphy287@charter.net</t>
   </si>
 </sst>
 </file>
@@ -624,7 +762,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A2F97E2D-D2EE-4E19-AA28-ED70E4256082}">
-  <dimension ref="A1:E43"/>
+  <dimension ref="A1:E56"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="27.5703125" customWidth="1"/>
@@ -694,10 +832,13 @@
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>11</v>
+        <v>85</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>86</v>
       </c>
       <c r="C5" s="1">
-        <v>1970</v>
+        <v>1987</v>
       </c>
       <c r="D5" t="b">
         <v>1</v>
@@ -705,10 +846,13 @@
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>10</v>
+        <v>11</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>91</v>
       </c>
       <c r="C6" s="1">
-        <v>1981</v>
+        <v>1970</v>
       </c>
       <c r="D6" t="b">
         <v>1</v>
@@ -716,13 +860,10 @@
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>8</v>
-      </c>
-      <c r="B7" t="s">
-        <v>56</v>
+        <v>10</v>
       </c>
       <c r="C7" s="1">
-        <v>1970</v>
+        <v>1981</v>
       </c>
       <c r="D7" t="b">
         <v>1</v>
@@ -730,10 +871,13 @@
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>5</v>
-      </c>
-      <c r="C8" s="1" t="s">
-        <v>21</v>
+        <v>87</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="C8" s="1">
+        <v>2995</v>
       </c>
       <c r="D8" t="b">
         <v>1</v>
@@ -741,30 +885,27 @@
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>30</v>
-      </c>
-      <c r="B9" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>21</v>
+        <v>8</v>
+      </c>
+      <c r="B9" t="s">
+        <v>56</v>
+      </c>
+      <c r="C9" s="1">
+        <v>1970</v>
       </c>
       <c r="D9" t="b">
-        <v>1</v>
-      </c>
-      <c r="E9" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>51</v>
-      </c>
-      <c r="B10" s="3" t="s">
-        <v>52</v>
-      </c>
-      <c r="C10" s="1">
-        <v>1989</v>
+        <v>5</v>
+      </c>
+      <c r="B10" t="s">
+        <v>92</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>21</v>
       </c>
       <c r="D10" t="b">
         <v>1</v>
@@ -772,39 +913,44 @@
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>61</v>
+        <v>30</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>62</v>
-      </c>
-      <c r="C11" s="1">
-        <v>1969</v>
+        <v>31</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>21</v>
       </c>
       <c r="D11" t="b">
+        <v>1</v>
+      </c>
+      <c r="E11" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>6</v>
+        <v>51</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="C12" s="1" t="s">
-        <v>21</v>
+        <v>52</v>
+      </c>
+      <c r="C12" s="1">
+        <v>1989</v>
       </c>
       <c r="D12" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A13" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="B13" s="2"/>
+      <c r="A13" t="s">
+        <v>61</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>62</v>
+      </c>
       <c r="C13" s="1">
-        <v>1982</v>
+        <v>1969</v>
       </c>
       <c r="D13" t="b">
         <v>1</v>
@@ -812,21 +958,27 @@
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>16</v>
-      </c>
-      <c r="C14" s="1">
-        <v>1964</v>
+        <v>6</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>21</v>
       </c>
       <c r="D14" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
-        <v>0</v>
+      <c r="A15" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>93</v>
       </c>
       <c r="C15" s="1">
-        <v>1969</v>
+        <v>1982</v>
       </c>
       <c r="D15" t="b">
         <v>1</v>
@@ -834,13 +986,13 @@
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>43</v>
-      </c>
-      <c r="B16" s="3" t="s">
-        <v>44</v>
-      </c>
-      <c r="C16" s="1" t="s">
-        <v>21</v>
+        <v>16</v>
+      </c>
+      <c r="B16" t="s">
+        <v>94</v>
+      </c>
+      <c r="C16" s="1">
+        <v>1964</v>
       </c>
       <c r="D16" t="b">
         <v>1</v>
@@ -848,10 +1000,13 @@
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>24</v>
+        <v>0</v>
+      </c>
+      <c r="B17" s="3" t="s">
+        <v>95</v>
       </c>
       <c r="C17" s="1">
-        <v>1979</v>
+        <v>1969</v>
       </c>
       <c r="D17" t="b">
         <v>1</v>
@@ -859,10 +1014,13 @@
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>4</v>
-      </c>
-      <c r="C18" s="1">
-        <v>1971</v>
+        <v>43</v>
+      </c>
+      <c r="B18" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="C18" s="1" t="s">
+        <v>21</v>
       </c>
       <c r="D18" t="b">
         <v>1</v>
@@ -870,10 +1028,13 @@
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>19</v>
+        <v>24</v>
+      </c>
+      <c r="B19" t="s">
+        <v>96</v>
       </c>
       <c r="C19" s="1">
-        <v>1972</v>
+        <v>1979</v>
       </c>
       <c r="D19" t="b">
         <v>1</v>
@@ -881,24 +1042,27 @@
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>64</v>
-      </c>
-      <c r="B20" s="3" t="s">
-        <v>65</v>
+        <v>4</v>
+      </c>
+      <c r="B20" t="s">
+        <v>97</v>
       </c>
       <c r="C20" s="1">
-        <v>1979</v>
+        <v>1971</v>
       </c>
       <c r="D20" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>20</v>
+        <v>72</v>
+      </c>
+      <c r="B21" s="3" t="s">
+        <v>73</v>
       </c>
       <c r="C21" s="1">
-        <v>1979</v>
+        <v>1993</v>
       </c>
       <c r="D21" t="b">
         <v>1</v>
@@ -906,10 +1070,13 @@
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>28</v>
+        <v>19</v>
+      </c>
+      <c r="B22" t="s">
+        <v>98</v>
       </c>
       <c r="C22" s="1">
-        <v>1982</v>
+        <v>1972</v>
       </c>
       <c r="D22" t="b">
         <v>1</v>
@@ -917,10 +1084,13 @@
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>2</v>
+        <v>64</v>
+      </c>
+      <c r="B23" s="3" t="s">
+        <v>65</v>
       </c>
       <c r="C23" s="1">
-        <v>1987</v>
+        <v>1979</v>
       </c>
       <c r="D23" t="b">
         <v>1</v>
@@ -928,10 +1098,13 @@
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>26</v>
+        <v>20</v>
+      </c>
+      <c r="B24" t="s">
+        <v>99</v>
       </c>
       <c r="C24" s="1">
-        <v>1986</v>
+        <v>1979</v>
       </c>
       <c r="D24" t="b">
         <v>1</v>
@@ -939,13 +1112,13 @@
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>48</v>
+        <v>83</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>49</v>
+        <v>84</v>
       </c>
       <c r="C25" s="1">
-        <v>1966</v>
+        <v>1986</v>
       </c>
       <c r="D25" t="b">
         <v>1</v>
@@ -953,10 +1126,13 @@
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>25</v>
+        <v>28</v>
+      </c>
+      <c r="B26" s="3" t="s">
+        <v>100</v>
       </c>
       <c r="C26" s="1">
-        <v>1979</v>
+        <v>1982</v>
       </c>
       <c r="D26" t="b">
         <v>1</v>
@@ -964,10 +1140,13 @@
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>1</v>
-      </c>
-      <c r="C27" s="1">
-        <v>1970</v>
+        <v>76</v>
+      </c>
+      <c r="B27" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="C27" s="1" t="s">
+        <v>21</v>
       </c>
       <c r="D27" t="b">
         <v>1</v>
@@ -975,10 +1154,13 @@
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>3</v>
+        <v>2</v>
+      </c>
+      <c r="B28" t="s">
+        <v>101</v>
       </c>
       <c r="C28" s="1">
-        <v>2015</v>
+        <v>1987</v>
       </c>
       <c r="D28" t="b">
         <v>1</v>
@@ -986,13 +1168,13 @@
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>66</v>
+        <v>78</v>
       </c>
       <c r="B29" s="3" t="s">
-        <v>67</v>
+        <v>79</v>
       </c>
       <c r="C29" s="1">
-        <v>1978</v>
+        <v>1981</v>
       </c>
       <c r="D29" t="b">
         <v>1</v>
@@ -1000,10 +1182,13 @@
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>7</v>
+        <v>104</v>
+      </c>
+      <c r="B30" s="3" t="s">
+        <v>105</v>
       </c>
       <c r="C30" s="1">
-        <v>1969</v>
+        <v>1981</v>
       </c>
       <c r="D30" t="b">
         <v>1</v>
@@ -1011,13 +1196,13 @@
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>15</v>
-      </c>
-      <c r="B31" s="3" t="s">
-        <v>50</v>
+        <v>26</v>
+      </c>
+      <c r="B31" t="s">
+        <v>102</v>
       </c>
       <c r="C31" s="1">
-        <v>1971</v>
+        <v>1986</v>
       </c>
       <c r="D31" t="b">
         <v>1</v>
@@ -1025,10 +1210,13 @@
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>12</v>
-      </c>
-      <c r="C32" s="1" t="s">
-        <v>21</v>
+        <v>48</v>
+      </c>
+      <c r="B32" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="C32" s="1">
+        <v>1966</v>
       </c>
       <c r="D32" t="b">
         <v>1</v>
@@ -1036,13 +1224,13 @@
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>37</v>
+        <v>112</v>
       </c>
       <c r="B33" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="C33" s="1" t="s">
-        <v>21</v>
+        <v>113</v>
+      </c>
+      <c r="C33" s="1">
+        <v>1992</v>
       </c>
       <c r="D33" t="b">
         <v>1</v>
@@ -1050,13 +1238,13 @@
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>39</v>
+        <v>89</v>
       </c>
       <c r="B34" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="C34" s="1" t="s">
-        <v>21</v>
+        <v>90</v>
+      </c>
+      <c r="C34" s="1">
+        <v>1984</v>
       </c>
       <c r="D34" t="b">
         <v>1</v>
@@ -1064,10 +1252,13 @@
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>13</v>
+        <v>68</v>
+      </c>
+      <c r="B35" s="3" t="s">
+        <v>69</v>
       </c>
       <c r="C35" s="1">
-        <v>1970</v>
+        <v>1979</v>
       </c>
       <c r="D35" t="b">
         <v>1</v>
@@ -1075,13 +1266,13 @@
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>22</v>
-      </c>
-      <c r="B36" s="3" t="s">
-        <v>63</v>
+        <v>25</v>
+      </c>
+      <c r="B36" t="s">
+        <v>103</v>
       </c>
       <c r="C36" s="1">
-        <v>1975</v>
+        <v>1979</v>
       </c>
       <c r="D36" t="b">
         <v>1</v>
@@ -1089,13 +1280,13 @@
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>41</v>
-      </c>
-      <c r="B37" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="C37" s="1" t="s">
-        <v>21</v>
+        <v>1</v>
+      </c>
+      <c r="B37" t="s">
+        <v>106</v>
+      </c>
+      <c r="C37" s="1">
+        <v>1970</v>
       </c>
       <c r="D37" t="b">
         <v>1</v>
@@ -1103,13 +1294,13 @@
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>45</v>
-      </c>
-      <c r="B38" s="3" t="s">
-        <v>46</v>
+        <v>3</v>
+      </c>
+      <c r="B38" t="s">
+        <v>107</v>
       </c>
       <c r="C38" s="1">
-        <v>1970</v>
+        <v>2015</v>
       </c>
       <c r="D38" t="b">
         <v>1</v>
@@ -1117,10 +1308,13 @@
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>17</v>
+        <v>66</v>
+      </c>
+      <c r="B39" s="3" t="s">
+        <v>67</v>
       </c>
       <c r="C39" s="1">
-        <v>1969</v>
+        <v>1978</v>
       </c>
       <c r="D39" t="b">
         <v>1</v>
@@ -1128,10 +1322,13 @@
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>9</v>
-      </c>
-      <c r="C40" s="1" t="s">
-        <v>21</v>
+        <v>70</v>
+      </c>
+      <c r="B40" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="C40" s="1">
+        <v>1974</v>
       </c>
       <c r="D40" t="b">
         <v>1</v>
@@ -1139,10 +1336,13 @@
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>23</v>
+        <v>7</v>
+      </c>
+      <c r="B41" t="s">
+        <v>108</v>
       </c>
       <c r="C41" s="1">
-        <v>1979</v>
+        <v>1969</v>
       </c>
       <c r="D41" t="b">
         <v>1</v>
@@ -1150,13 +1350,13 @@
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>57</v>
+        <v>82</v>
       </c>
       <c r="B42" s="3" t="s">
-        <v>58</v>
+        <v>81</v>
       </c>
       <c r="C42" s="1">
-        <v>2006</v>
+        <v>1968</v>
       </c>
       <c r="D42" t="b">
         <v>1</v>
@@ -1164,40 +1364,237 @@
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
+        <v>15</v>
+      </c>
+      <c r="B43" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="C43" s="1">
+        <v>1971</v>
+      </c>
+      <c r="D43" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>12</v>
+      </c>
+      <c r="B44" s="3" t="s">
+        <v>109</v>
+      </c>
+      <c r="C44" s="1">
+        <v>1985</v>
+      </c>
+      <c r="D44" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>37</v>
+      </c>
+      <c r="B45" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="C45" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D45" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>39</v>
+      </c>
+      <c r="B46" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="C46" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D46" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>13</v>
+      </c>
+      <c r="B47" t="s">
+        <v>110</v>
+      </c>
+      <c r="C47" s="1">
+        <v>1970</v>
+      </c>
+      <c r="D47" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
+        <v>22</v>
+      </c>
+      <c r="B48" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="C48" s="1">
+        <v>1975</v>
+      </c>
+      <c r="D48" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>41</v>
+      </c>
+      <c r="B49" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="C49" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D49" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>45</v>
+      </c>
+      <c r="B50" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="C50" s="1">
+        <v>1970</v>
+      </c>
+      <c r="D50" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>17</v>
+      </c>
+      <c r="B51" t="s">
+        <v>111</v>
+      </c>
+      <c r="C51" s="1">
+        <v>1969</v>
+      </c>
+      <c r="D51" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
+        <v>74</v>
+      </c>
+      <c r="B52" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="C52" s="1">
+        <v>1975</v>
+      </c>
+      <c r="D52" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A53" t="s">
+        <v>9</v>
+      </c>
+      <c r="B53" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="C53" s="1">
+        <v>1989</v>
+      </c>
+      <c r="D53" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="54" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A54" t="s">
+        <v>23</v>
+      </c>
+      <c r="C54" s="1">
+        <v>1979</v>
+      </c>
+      <c r="D54" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="55" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A55" t="s">
+        <v>57</v>
+      </c>
+      <c r="B55" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="C55" s="1">
+        <v>2006</v>
+      </c>
+      <c r="D55" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="56" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A56" t="s">
         <v>53</v>
       </c>
-      <c r="B43" s="3" t="s">
+      <c r="B56" s="3" t="s">
         <v>54</v>
       </c>
-      <c r="C43" s="1">
+      <c r="C56" s="1">
         <v>1975</v>
       </c>
-      <c r="D43" t="b">
+      <c r="D56" t="b">
         <v>1</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="B4" r:id="rId1" xr:uid="{8227A597-9225-4357-B8B6-9F19CC6D2D47}"/>
-    <hyperlink ref="B9" r:id="rId2" display="mailto:Rxbras@gmail.com" xr:uid="{C440EE30-529A-4080-AE83-A4A978C3E02B}"/>
-    <hyperlink ref="B33" r:id="rId3" display="mailto:christopher.pavasaris@gmail.com" xr:uid="{C5FAAB38-5F1C-4A08-8709-401E7E23E0D1}"/>
-    <hyperlink ref="B34" r:id="rId4" display="mailto:hll.reed01@gmail.com" xr:uid="{109EA93A-660A-4099-B212-FD77BC4B5297}"/>
-    <hyperlink ref="B37" r:id="rId5" display="mailto:adam@odysseyteencamp.com" xr:uid="{4FC29F3F-346D-4C86-81DD-BA31CA08B134}"/>
-    <hyperlink ref="B16" r:id="rId6" display="mailto:michael.estep@acps.k12.va.us" xr:uid="{98703E9F-F4A5-4829-8BBF-B9F807C63E68}"/>
-    <hyperlink ref="B38" r:id="rId7" display="mailto:1photodog@gmail.com" xr:uid="{9E8BA56C-3438-4645-83BE-2770570162B4}"/>
-    <hyperlink ref="B12" r:id="rId8" display="mailto:artchristiani@gmail.com" xr:uid="{804D2DB9-BDF1-463B-9BD3-ACBFC15F041A}"/>
-    <hyperlink ref="B25" r:id="rId9" display="mailto:Jlmorgan3@icloud.com" xr:uid="{03952628-4855-439F-9B40-CAC6626447C4}"/>
-    <hyperlink ref="B31" r:id="rId10" display="mailto:npisciottano@hotmail.com" xr:uid="{781976BA-4287-4FD4-8728-D3D09F930C18}"/>
-    <hyperlink ref="B10" r:id="rId11" display="mailto:bcarignan85@gmail.com" xr:uid="{DF6F8079-E647-4079-9719-72DC2FF3791C}"/>
-    <hyperlink ref="B43" r:id="rId12" display="mailto:martha529@aol.com" xr:uid="{6DF6CCA4-C8CA-41C8-BD42-527DBB5CB505}"/>
-    <hyperlink ref="B42" r:id="rId13" display="mailto:jason.derek.ward@gmail.com" xr:uid="{ECCFE763-5E69-4122-B27B-DA1C21FADA86}"/>
+    <hyperlink ref="B11" r:id="rId2" xr:uid="{C440EE30-529A-4080-AE83-A4A978C3E02B}"/>
+    <hyperlink ref="B45" r:id="rId3" xr:uid="{C5FAAB38-5F1C-4A08-8709-401E7E23E0D1}"/>
+    <hyperlink ref="B46" r:id="rId4" xr:uid="{109EA93A-660A-4099-B212-FD77BC4B5297}"/>
+    <hyperlink ref="B49" r:id="rId5" xr:uid="{4FC29F3F-346D-4C86-81DD-BA31CA08B134}"/>
+    <hyperlink ref="B18" r:id="rId6" xr:uid="{98703E9F-F4A5-4829-8BBF-B9F807C63E68}"/>
+    <hyperlink ref="B50" r:id="rId7" display="mailto:1photodog@gmail.com" xr:uid="{9E8BA56C-3438-4645-83BE-2770570162B4}"/>
+    <hyperlink ref="B14" r:id="rId8" xr:uid="{804D2DB9-BDF1-463B-9BD3-ACBFC15F041A}"/>
+    <hyperlink ref="B32" r:id="rId9" xr:uid="{03952628-4855-439F-9B40-CAC6626447C4}"/>
+    <hyperlink ref="B43" r:id="rId10" display="mailto:npisciottano@hotmail.com" xr:uid="{781976BA-4287-4FD4-8728-D3D09F930C18}"/>
+    <hyperlink ref="B12" r:id="rId11" xr:uid="{DF6F8079-E647-4079-9719-72DC2FF3791C}"/>
+    <hyperlink ref="B56" r:id="rId12" xr:uid="{6DF6CCA4-C8CA-41C8-BD42-527DBB5CB505}"/>
+    <hyperlink ref="B55" r:id="rId13" xr:uid="{ECCFE763-5E69-4122-B27B-DA1C21FADA86}"/>
     <hyperlink ref="B2" r:id="rId14" display="mailto:louabare@yahoo.com" xr:uid="{8869974B-11E2-4A99-8438-9F9B8ABEB9F6}"/>
-    <hyperlink ref="B11" r:id="rId15" display="mailto:elizabeth.casarella@gmail.com" xr:uid="{C150E814-8C96-4E50-8A55-5EB3344749B1}"/>
-    <hyperlink ref="B36" r:id="rId16" display="mailto:paul@levelbreaker.com" xr:uid="{9746CC3F-863E-4E18-931A-FADD4ED10BF2}"/>
-    <hyperlink ref="B20" r:id="rId17" display="mailto:Drjpkonecny@gmail.com" xr:uid="{316BCF75-05DF-4572-9F46-9F76127C0677}"/>
-    <hyperlink ref="B29" r:id="rId18" display="mailto:dennis.p.oconnell@gmail.com" xr:uid="{57197F8F-1C51-4977-936A-74B15D239DF7}"/>
+    <hyperlink ref="B13" r:id="rId15" display="mailto:elizabeth.casarella@gmail.com" xr:uid="{C150E814-8C96-4E50-8A55-5EB3344749B1}"/>
+    <hyperlink ref="B48" r:id="rId16" display="mailto:paul@levelbreaker.com" xr:uid="{9746CC3F-863E-4E18-931A-FADD4ED10BF2}"/>
+    <hyperlink ref="B23" r:id="rId17" xr:uid="{316BCF75-05DF-4572-9F46-9F76127C0677}"/>
+    <hyperlink ref="B39" r:id="rId18" display="mailto:dennis.p.oconnell@gmail.com" xr:uid="{57197F8F-1C51-4977-936A-74B15D239DF7}"/>
+    <hyperlink ref="B35" r:id="rId19" display="mailto:hef714@aol.com" xr:uid="{A4825BC7-F2DD-43E9-A39B-48544C54E403}"/>
+    <hyperlink ref="B40" r:id="rId20" xr:uid="{53A4A1D2-46D5-45C1-BB62-DA92169DD070}"/>
+    <hyperlink ref="B21" r:id="rId21" xr:uid="{A871275A-577B-4F01-A590-B30FBADA40A1}"/>
+    <hyperlink ref="B52" r:id="rId22" xr:uid="{7E7AC9EC-4484-43DC-8B81-7AA0BCCFA407}"/>
+    <hyperlink ref="B29" r:id="rId23" display="mailto:Gjhusky52@yahoo.com" xr:uid="{1F5D9E16-5BA9-4F8F-B8CF-14485F325E5D}"/>
+    <hyperlink ref="B53" r:id="rId24" display="mailto:s.vibberts@yahoo.com" xr:uid="{CD95CA65-C8C5-44B3-8AFC-2E088AEC194C}"/>
+    <hyperlink ref="B42" r:id="rId25" display="mailto:oldparsonage3@gmail.com" xr:uid="{DC8DA8C9-CCEA-4FC3-AA05-1EF34B65B0C1}"/>
+    <hyperlink ref="B25" r:id="rId26" xr:uid="{C2395B48-B35E-4045-A136-C8B31BE4A5FC}"/>
+    <hyperlink ref="B5" r:id="rId27" display="mailto:patrick@drpflexpak.com" xr:uid="{37F7977A-EC68-4733-8738-6C53C959B816}"/>
+    <hyperlink ref="B8" r:id="rId28" display="mailto:cwb84122@gmail.com" xr:uid="{A209B655-7CEF-4F8D-BFEE-DFB49C33870B}"/>
+    <hyperlink ref="B34" r:id="rId29" display="mailto:Npmyers@sbcglobal.net" xr:uid="{46F1EE8C-941D-4D6B-A27A-3BDDA65A15CE}"/>
+    <hyperlink ref="B6" r:id="rId30" xr:uid="{647703FF-1796-4612-923D-2A3CF89F5A46}"/>
+    <hyperlink ref="B17" r:id="rId31" xr:uid="{D4F421DD-A322-4F00-A209-B464A28664A6}"/>
+    <hyperlink ref="B26" r:id="rId32" xr:uid="{5FF15619-CFAB-48CB-8BF0-78013919701C}"/>
+    <hyperlink ref="B30" r:id="rId33" display="mailto:Kmills8080@gmail.com" xr:uid="{6653A4F2-00C8-4ACF-A9B2-950ABB23037C}"/>
+    <hyperlink ref="B27" r:id="rId34" xr:uid="{0F8932AA-3F92-4F04-A82F-C839649C3558}"/>
+    <hyperlink ref="B44" r:id="rId35" xr:uid="{74573551-A238-45F0-95FA-078470676D33}"/>
+    <hyperlink ref="B33" r:id="rId36" xr:uid="{F093A50A-9255-43F2-873A-E61FB97B7B6E}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId19"/>
+  <pageSetup orientation="portrait" r:id="rId37"/>
 </worksheet>
 </file>
</xml_diff>